<commit_message>
quitar columna emojis en db y adaptar toda la pagina al igual que las importaciones de categorias
</commit_message>
<xml_diff>
--- a/public/plantilla_categorias.xlsx
+++ b/public/plantilla_categorias.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Categorías" sheetId="1" r:id="rId4"/>
+    <sheet name="Categorias" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -26,64 +26,94 @@
     <t>description</t>
   </si>
   <si>
-    <t>icono_emoji</t>
-  </si>
-  <si>
-    <t>Celulares y Smartphones</t>
-  </si>
-  <si>
-    <t>celulares</t>
-  </si>
-  <si>
-    <t>Teléfonos móviles y accesorios</t>
-  </si>
-  <si>
-    <t>📱</t>
-  </si>
-  <si>
-    <t>Computadoras y Laptops</t>
-  </si>
-  <si>
-    <t>computadoras</t>
-  </si>
-  <si>
-    <t>PCs, laptops y periféricos</t>
-  </si>
-  <si>
-    <t>💻</t>
-  </si>
-  <si>
-    <t>Audio y Sonido</t>
-  </si>
-  <si>
-    <t>audio</t>
-  </si>
-  <si>
-    <t>Parlantes, auriculares y equipos de audio</t>
-  </si>
-  <si>
-    <t>🔊</t>
-  </si>
-  <si>
-    <t>TV y Video</t>
-  </si>
-  <si>
-    <t>tv-video</t>
-  </si>
-  <si>
-    <t>Televisores y reproductores</t>
-  </si>
-  <si>
-    <t>📺</t>
-  </si>
-  <si>
-    <t>Cámaras y Fotografía</t>
-  </si>
-  <si>
-    <t>Cámaras digitales y accesorios</t>
-  </si>
-  <si>
-    <t>📷</t>
+    <t>Electronica</t>
+  </si>
+  <si>
+    <t>electronica</t>
+  </si>
+  <si>
+    <t>Todos los dispositivos electronicos</t>
+  </si>
+  <si>
+    <t>Computacion</t>
+  </si>
+  <si>
+    <t>computacion</t>
+  </si>
+  <si>
+    <t>Computadoras laptops y accesorios</t>
+  </si>
+  <si>
+    <t>Audio Video</t>
+  </si>
+  <si>
+    <t>audio-video</t>
+  </si>
+  <si>
+    <t>Auriculares parlantes y monitores</t>
+  </si>
+  <si>
+    <t>Accesorios</t>
+  </si>
+  <si>
+    <t>accesorios</t>
+  </si>
+  <si>
+    <t>Cables cargadores y perifericos</t>
+  </si>
+  <si>
+    <t>Smartphones</t>
+  </si>
+  <si>
+    <t>smartphones</t>
+  </si>
+  <si>
+    <t>Celulares y accesorios</t>
+  </si>
+  <si>
+    <t>Tablets</t>
+  </si>
+  <si>
+    <t>tablets</t>
+  </si>
+  <si>
+    <t>Tablets y accesorios</t>
+  </si>
+  <si>
+    <t>Gaming</t>
+  </si>
+  <si>
+    <t>gaming</t>
+  </si>
+  <si>
+    <t>Equipos y accesorios para juegos</t>
+  </si>
+  <si>
+    <t>Redes</t>
+  </si>
+  <si>
+    <t>redes</t>
+  </si>
+  <si>
+    <t>Routers switches y equipamiento de red</t>
+  </si>
+  <si>
+    <t>Almacenamiento</t>
+  </si>
+  <si>
+    <t>almacenamiento</t>
+  </si>
+  <si>
+    <t>Discos USB y memorias</t>
+  </si>
+  <si>
+    <t>Componentes</t>
+  </si>
+  <si>
+    <t>componentes</t>
+  </si>
+  <si>
+    <t>Partes y piezas para PC</t>
   </si>
 </sst>
 </file>
@@ -91,7 +121,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -101,28 +131,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1a1a2e"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -137,11 +152,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,95 +453,128 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="49.417" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16.282" bestFit="true" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="B6"/>
-      <c r="C6" t="s">
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="D6" t="s">
+      <c r="B8" t="s">
         <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>